<commit_message>
eloqwnt: refresh AI workbook after SERP intent check
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/eloqwnt/keyword-research-ai.xlsx
+++ b/decks/eloqwnt/keyword-research-ai.xlsx
@@ -552,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="J3" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -1373,23 +1373,23 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Subscription Based Website: What to Expect &amp; Pricing</t>
+          <t>Low Cost Website Design: What to Expect &amp; Pricing</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>subscription based website</t>
+          <t>low cost website design</t>
         </is>
       </c>
       <c r="D19" s="4" t="n">
         <v>260</v>
       </c>
       <c r="E19" t="n">
-        <v>20</v>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>40</v>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
@@ -1417,19 +1417,19 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Low Cost Website Design: A Smarter Way to Brief It</t>
+          <t>Unlimited Design Service: Faster, Leaner, Smarter</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>low cost website design</t>
+          <t>unlimited design service</t>
         </is>
       </c>
       <c r="D20" s="4" t="n">
-        <v>260</v>
+        <v>210</v>
       </c>
       <c r="E20" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
@@ -1461,23 +1461,23 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Subscription Website: Speed, Scope &amp; Budget</t>
+          <t>Graphic Design Monthly Subscription Without the Agency Price Tag</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>subscription website</t>
+          <t>graphic design monthly subscription</t>
         </is>
       </c>
       <c r="D21" s="4" t="n">
         <v>210</v>
       </c>
       <c r="E21" t="n">
-        <v>20</v>
-      </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>49</v>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G21" s="10" t="inlineStr">
@@ -1505,23 +1505,23 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Unlimited Design Service Without the Agency Price Tag</t>
+          <t>Unlimited Graphic Design Packages: How AI Cuts Cost, Not Quality</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>unlimited design service</t>
+          <t>unlimited graphic design packages</t>
         </is>
       </c>
       <c r="D22" s="4" t="n">
         <v>210</v>
       </c>
       <c r="E22" t="n">
-        <v>38</v>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>50</v>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>Hard</t>
         </is>
       </c>
       <c r="G22" s="10" t="inlineStr">
@@ -1536,7 +1536,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="J22" s="2" t="n">
@@ -1549,23 +1549,23 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Graphic Design Monthly Subscription: What to Expect &amp; Pricing</t>
+          <t>On Demand Graphic Design: Speed, Scope &amp; Budget</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>graphic design monthly subscription</t>
+          <t>on demand graphic design</t>
         </is>
       </c>
       <c r="D23" s="4" t="n">
-        <v>210</v>
+        <v>170</v>
       </c>
       <c r="E23" t="n">
-        <v>49</v>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>18</v>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G23" s="10" t="inlineStr">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="J23" s="2" t="n">
@@ -1593,23 +1593,23 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Unlimited Graphic Design Packages: Speed, Scope &amp; Budget</t>
+          <t>Web Design Subscription: A Smarter Way to Brief It</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>unlimited graphic design packages</t>
+          <t>web design subscription</t>
         </is>
       </c>
       <c r="D24" s="4" t="n">
-        <v>210</v>
+        <v>170</v>
       </c>
       <c r="E24" t="n">
-        <v>50</v>
-      </c>
-      <c r="F24" s="12" t="inlineStr">
-        <is>
-          <t>Hard</t>
+        <v>18</v>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G24" s="10" t="inlineStr">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Bottom of funnel</t>
         </is>
       </c>
       <c r="J24" s="2" t="n">
@@ -1637,23 +1637,23 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>On Demand Graphic Design: Faster, Leaner, Smarter</t>
+          <t>Subscription Design Services: What to Expect &amp; Pricing</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>on demand graphic design</t>
+          <t>subscription design services</t>
         </is>
       </c>
       <c r="D25" s="4" t="n">
-        <v>170</v>
+        <v>140</v>
       </c>
       <c r="E25" t="n">
-        <v>18</v>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>39</v>
+      </c>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G25" s="10" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Bottom of funnel</t>
         </is>
       </c>
       <c r="J25" s="2" t="n">
@@ -1681,23 +1681,23 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Web Design Subscription: Quality on a Faster Timeline</t>
+          <t>Unlimited Design Subscription: A Smarter Way to Brief It</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>web design subscription</t>
+          <t>unlimited design subscription</t>
         </is>
       </c>
       <c r="D26" s="4" t="n">
-        <v>170</v>
+        <v>140</v>
       </c>
       <c r="E26" t="n">
-        <v>18</v>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>44</v>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G26" s="10" t="inlineStr">
@@ -1725,19 +1725,19 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Subscription Design Services: A Smarter Way to Brief It</t>
+          <t>Low Cost Logo Design: Faster, Leaner, Smarter</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>subscription design services</t>
+          <t>low cost logo design</t>
         </is>
       </c>
       <c r="D27" s="4" t="n">
         <v>140</v>
       </c>
       <c r="E27" t="n">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -1769,23 +1769,23 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Unlimited Design Subscription: Quality on a Faster Timeline</t>
+          <t>Affordable Branding Agency: Quality on a Faster Timeline</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>unlimited design subscription</t>
+          <t>affordable branding agency</t>
         </is>
       </c>
       <c r="D28" s="4" t="n">
-        <v>140</v>
+        <v>110</v>
       </c>
       <c r="E28" t="n">
-        <v>44</v>
-      </c>
-      <c r="F28" s="9" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>10</v>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G28" s="10" t="inlineStr">
@@ -1813,23 +1813,23 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Low Cost Logo Design Without the Agency Price Tag</t>
+          <t>Product Design Subscription: What to Expect &amp; Pricing</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>low cost logo design</t>
+          <t>product design subscription</t>
         </is>
       </c>
       <c r="D29" s="4" t="n">
-        <v>140</v>
+        <v>110</v>
       </c>
       <c r="E29" t="n">
-        <v>49</v>
-      </c>
-      <c r="F29" s="9" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>15</v>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G29" s="10" t="inlineStr">
@@ -1857,23 +1857,23 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Affordable Branding Agency: How AI Cuts Cost, Not Quality</t>
+          <t>Unlimited Web Development: Speed, Scope &amp; Budget</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>affordable branding agency</t>
+          <t>unlimited web development</t>
         </is>
       </c>
       <c r="D30" s="4" t="n">
         <v>110</v>
       </c>
       <c r="E30" t="n">
-        <v>10</v>
-      </c>
-      <c r="F30" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>17</v>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G30" s="10" t="inlineStr">
@@ -1888,7 +1888,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="J30" s="2" t="n">
@@ -1901,19 +1901,19 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Product Design Subscription: A Smarter Way to Brief It</t>
+          <t>Subscription Based Design Services Without the Agency Price Tag</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>product design subscription</t>
+          <t>subscription based design services</t>
         </is>
       </c>
       <c r="D31" s="4" t="n">
         <v>110</v>
       </c>
       <c r="E31" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
@@ -1945,19 +1945,19 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Unlimited Web Development: Faster, Leaner, Smarter</t>
+          <t>Affordable Graphic Design Services: Speed, Scope &amp; Budget</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>unlimited web development</t>
+          <t>affordable graphic design services</t>
         </is>
       </c>
       <c r="D32" s="4" t="n">
         <v>110</v>
       </c>
       <c r="E32" t="n">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
@@ -1976,7 +1976,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Bottom of funnel</t>
         </is>
       </c>
       <c r="J32" s="2" t="n">
@@ -1989,23 +1989,23 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Subscription Based Design Services: What to Expect &amp; Pricing</t>
+          <t>Design Subscription Agency: Quality on a Faster Timeline</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>subscription based design services</t>
+          <t>design subscription agency</t>
         </is>
       </c>
       <c r="D33" s="4" t="n">
         <v>110</v>
       </c>
       <c r="E33" t="n">
-        <v>25</v>
-      </c>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>35</v>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G33" s="10" t="inlineStr">
@@ -2033,23 +2033,23 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Affordable Graphic Design Services: Faster, Leaner, Smarter</t>
+          <t>Unlimited Graphic Design for Monthly Fee Without the Agency Price Tag</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>affordable graphic design services</t>
+          <t>unlimited graphic design for monthly fee</t>
         </is>
       </c>
       <c r="D34" s="4" t="n">
         <v>110</v>
       </c>
       <c r="E34" t="n">
-        <v>29</v>
-      </c>
-      <c r="F34" s="5" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>36</v>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G34" s="10" t="inlineStr">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="J34" s="2" t="n">
@@ -2077,23 +2077,23 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Design Subscription Agency: What to Expect &amp; Pricing</t>
+          <t>Graphic Design Subscription Service: How AI Cuts Cost, Not Quality</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>design subscription agency</t>
+          <t>graphic design subscription service</t>
         </is>
       </c>
       <c r="D35" s="4" t="n">
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="E35" t="n">
-        <v>35</v>
-      </c>
-      <c r="F35" s="9" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>16</v>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G35" s="10" t="inlineStr">
@@ -2121,19 +2121,19 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Unlimited Graphic Design for Monthly Fee: Speed, Scope &amp; Budget</t>
+          <t>Flat Rate Graphic Design Services: Speed, Scope &amp; Budget</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>unlimited graphic design for monthly fee</t>
+          <t>flat rate graphic design services</t>
         </is>
       </c>
       <c r="D36" s="4" t="n">
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="E36" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
@@ -2152,7 +2152,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Bottom of funnel</t>
         </is>
       </c>
       <c r="J36" s="2" t="n">
@@ -2165,23 +2165,23 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Graphic Design Subscription Service: Speed, Scope &amp; Budget</t>
+          <t>Best Quick Turnaround Design Services: A Smarter Way to Brief It</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>graphic design subscription service</t>
+          <t>best quick turnaround design services</t>
         </is>
       </c>
       <c r="D37" s="4" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="E37" t="n">
-        <v>16</v>
-      </c>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>3</v>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G37" s="10" t="inlineStr">
@@ -2209,23 +2209,23 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Flat Rate Graphic Design Services: Faster, Leaner, Smarter</t>
+          <t>Design Subscription for SaaS: Faster, Leaner, Smarter</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>flat rate graphic design services</t>
+          <t>design subscription for saas</t>
         </is>
       </c>
       <c r="D38" s="4" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="E38" t="n">
-        <v>32</v>
-      </c>
-      <c r="F38" s="9" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>4</v>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G38" s="10" t="inlineStr">
@@ -2253,19 +2253,19 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Best Quick Turnaround Design Services: Quality on a Faster Timeline</t>
+          <t>Affordable Branding Services: Quality on a Faster Timeline</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>best quick turnaround design services</t>
+          <t>affordable branding services</t>
         </is>
       </c>
       <c r="D39" s="4" t="n">
         <v>70</v>
       </c>
       <c r="E39" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F39" s="8" t="inlineStr">
         <is>
@@ -2297,23 +2297,23 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Design Subscription for SaaS Without the Agency Price Tag</t>
+          <t>Design as a Subscription: What to Expect &amp; Pricing</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>design subscription for saas</t>
+          <t>design as a subscription</t>
         </is>
       </c>
       <c r="D40" s="4" t="n">
         <v>70</v>
       </c>
       <c r="E40" t="n">
-        <v>4</v>
-      </c>
-      <c r="F40" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>17</v>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G40" s="10" t="inlineStr">
@@ -2341,23 +2341,23 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Affordable Branding Services: How AI Cuts Cost, Not Quality</t>
+          <t>Product and Web Design Subscription: A Smarter Way to Brief It</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>affordable branding services</t>
+          <t>product and web design subscription</t>
         </is>
       </c>
       <c r="D41" s="4" t="n">
         <v>70</v>
       </c>
       <c r="E41" t="n">
-        <v>6</v>
-      </c>
-      <c r="F41" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>32</v>
+      </c>
+      <c r="F41" s="9" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G41" s="10" t="inlineStr">
@@ -2385,23 +2385,23 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Design as a Subscription: A Smarter Way to Brief It</t>
+          <t>Unlimited Graphic Design Subscription: Faster, Leaner, Smarter</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>design as a subscription</t>
+          <t>unlimited graphic design subscription</t>
         </is>
       </c>
       <c r="D42" s="4" t="n">
         <v>70</v>
       </c>
       <c r="E42" t="n">
-        <v>17</v>
-      </c>
-      <c r="F42" s="5" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>42</v>
+      </c>
+      <c r="F42" s="9" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G42" s="10" t="inlineStr">
@@ -2429,19 +2429,19 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Product and Web Design Subscription: Quality on a Faster Timeline</t>
+          <t>Affordable Logo Design Packages: Quality on a Faster Timeline</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>product and web design subscription</t>
+          <t>affordable logo design packages</t>
         </is>
       </c>
       <c r="D43" s="4" t="n">
         <v>70</v>
       </c>
       <c r="E43" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
@@ -2460,7 +2460,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="J43" s="2" t="n">
@@ -2473,28 +2473,28 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Unlimited Graphic Design Subscription Without the Agency Price Tag</t>
+          <t>AI Logos vs a Real Brand Identity: What AI Gets Right (and Where a Studio Wins)</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>unlimited graphic design subscription</t>
+          <t>artificial intelligence logo</t>
         </is>
       </c>
       <c r="D44" s="4" t="n">
-        <v>70</v>
+        <v>1600</v>
       </c>
       <c r="E44" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="G44" s="10" t="inlineStr">
-        <is>
-          <t>Fast &amp; Affordable Design</t>
+      <c r="G44" s="13" t="inlineStr">
+        <is>
+          <t>AI + Human Thought Leadership</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="J44" s="2" t="n">
@@ -2517,28 +2517,28 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Affordable Logo Design Packages: What to Expect &amp; Pricing</t>
+          <t>AI in Branding: What It Means for Your Brand</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>affordable logo design packages</t>
+          <t>ai in branding</t>
         </is>
       </c>
       <c r="D45" s="4" t="n">
-        <v>70</v>
+        <v>140</v>
       </c>
       <c r="E45" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="G45" s="10" t="inlineStr">
-        <is>
-          <t>Fast &amp; Affordable Design</t>
+      <c r="G45" s="13" t="inlineStr">
+        <is>
+          <t>AI + Human Thought Leadership</t>
         </is>
       </c>
       <c r="H45" s="11" t="inlineStr">
@@ -2548,7 +2548,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="J45" s="2" t="n">
@@ -2561,23 +2561,23 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>AI Logos vs a Real Brand Identity: What AI Gets Right (and Where a Studio Wins)</t>
+          <t>AI vs Human Designers, Explained for B2B Teams</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>artificial intelligence logo</t>
+          <t>ai vs human designers</t>
         </is>
       </c>
       <c r="D46" s="4" t="n">
-        <v>1600</v>
+        <v>0</v>
       </c>
       <c r="E46" t="n">
-        <v>33</v>
-      </c>
-      <c r="F46" s="9" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>10</v>
+      </c>
+      <c r="F46" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G46" s="13" t="inlineStr">
@@ -2585,9 +2585,9 @@
           <t>AI + Human Thought Leadership</t>
         </is>
       </c>
-      <c r="H46" s="11" t="inlineStr">
-        <is>
-          <t>Demand now</t>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>Early-mover bet</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2596,7 +2596,7 @@
         </is>
       </c>
       <c r="J46" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47">
@@ -2605,23 +2605,23 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>AI in Branding: What It Means for Your Brand</t>
+          <t>Will AI Replace Web Designers? The B2B View</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>ai in branding</t>
+          <t>will ai replace web designers</t>
         </is>
       </c>
       <c r="D47" s="4" t="n">
-        <v>140</v>
+        <v>0</v>
       </c>
       <c r="E47" t="n">
-        <v>49</v>
-      </c>
-      <c r="F47" s="9" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>12</v>
+      </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G47" s="13" t="inlineStr">
@@ -2629,9 +2629,9 @@
           <t>AI + Human Thought Leadership</t>
         </is>
       </c>
-      <c r="H47" s="11" t="inlineStr">
-        <is>
-          <t>Demand now</t>
+      <c r="H47" s="7" t="inlineStr">
+        <is>
+          <t>Early-mover bet</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2640,7 +2640,7 @@
         </is>
       </c>
       <c r="J47" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48">
@@ -2649,23 +2649,23 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>AI vs Human Designers, Explained for B2B Teams</t>
+          <t>AI Design Trends to Watch in 2026</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>ai vs human designers</t>
+          <t>ai design trends 2026</t>
         </is>
       </c>
       <c r="D48" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E48" t="n">
-        <v>10</v>
-      </c>
-      <c r="F48" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>15</v>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G48" s="13" t="inlineStr">
@@ -2693,23 +2693,23 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Will AI Replace Web Designers? The B2B View</t>
+          <t>The Honest Take on AI and Graphic Design</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>will ai replace web designers</t>
+          <t>ai and graphic design</t>
         </is>
       </c>
       <c r="D49" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E49" t="n">
-        <v>12</v>
-      </c>
-      <c r="F49" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>20</v>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G49" s="13" t="inlineStr">
@@ -2737,23 +2737,23 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>AI Design Trends to Watch in 2026</t>
+          <t>The Future of Web Design Is AI + Human</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>ai design trends 2026</t>
+          <t>future of web design with ai</t>
         </is>
       </c>
       <c r="D50" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E50" t="n">
-        <v>15</v>
-      </c>
-      <c r="F50" s="5" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>12</v>
+      </c>
+      <c r="F50" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G50" s="13" t="inlineStr">
@@ -2781,23 +2781,23 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>The Honest Take on AI and Graphic Design</t>
+          <t>AI Impact on Branding for Design Leaders</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>ai and graphic design</t>
+          <t>ai impact on branding</t>
         </is>
       </c>
       <c r="D51" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E51" t="n">
-        <v>20</v>
-      </c>
-      <c r="F51" s="5" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>10</v>
+      </c>
+      <c r="F51" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G51" s="13" t="inlineStr">
@@ -2825,12 +2825,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>The Future of Web Design Is AI + Human</t>
+          <t>Human vs AI Design: A Practical 2026 View</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>future of web design with ai</t>
+          <t>human vs ai design</t>
         </is>
       </c>
       <c r="D52" s="4" t="n">
@@ -2869,23 +2869,23 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>AI Impact on Branding for Design Leaders</t>
+          <t>Rethinking AI Design Workflow for Modern Brands</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>ai impact on branding</t>
+          <t>ai design workflow</t>
         </is>
       </c>
       <c r="D53" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E53" t="n">
-        <v>10</v>
-      </c>
-      <c r="F53" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>18</v>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G53" s="13" t="inlineStr">
@@ -2913,19 +2913,19 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Human vs AI Design: A Practical 2026 View</t>
+          <t>AI for Design Agencies: What It Means for Your Brand</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>human vs ai design</t>
+          <t>ai for design agencies</t>
         </is>
       </c>
       <c r="D54" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E54" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F54" s="8" t="inlineStr">
         <is>
@@ -2957,23 +2957,23 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Rethinking AI Design Workflow for Modern Brands</t>
+          <t>AI Brand Strategy, Explained for B2B Teams</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>ai design workflow</t>
+          <t>ai brand strategy</t>
         </is>
       </c>
       <c r="D55" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E55" t="n">
-        <v>18</v>
-      </c>
-      <c r="F55" s="5" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>12</v>
+      </c>
+      <c r="F55" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G55" s="13" t="inlineStr">
@@ -3001,23 +3001,23 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>AI for Design Agencies: What It Means for Your Brand</t>
+          <t>The Honest Take on AI in UX Design</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>ai for design agencies</t>
+          <t>ai in ux design</t>
         </is>
       </c>
       <c r="D56" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E56" t="n">
-        <v>14</v>
-      </c>
-      <c r="F56" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>20</v>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G56" s="13" t="inlineStr">
@@ -3045,23 +3045,23 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>AI Brand Strategy, Explained for B2B Teams</t>
+          <t>Generative AI in Design: A Practical 2026 View</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>ai brand strategy</t>
+          <t>generative ai in design</t>
         </is>
       </c>
       <c r="D57" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E57" t="n">
-        <v>12</v>
-      </c>
-      <c r="F57" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>22</v>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G57" s="13" t="inlineStr">
@@ -3089,23 +3089,23 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>The Honest Take on AI in UX Design</t>
+          <t>Rethinking AI Augmented Design for Modern Brands</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>ai in ux design</t>
+          <t>ai augmented design</t>
         </is>
       </c>
       <c r="D58" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E58" t="n">
-        <v>20</v>
-      </c>
-      <c r="F58" s="5" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>12</v>
+      </c>
+      <c r="F58" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G58" s="13" t="inlineStr">
@@ -3133,19 +3133,19 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Generative AI in Design: A Practical 2026 View</t>
+          <t>Designing with AI for Design Leaders</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>generative ai in design</t>
+          <t>designing with ai</t>
         </is>
       </c>
       <c r="D59" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E59" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
@@ -3177,23 +3177,23 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Rethinking AI Augmented Design for Modern Brands</t>
+          <t>AI Design Process: What It Means for Your Brand</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>ai augmented design</t>
+          <t>ai design process</t>
         </is>
       </c>
       <c r="D60" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E60" t="n">
-        <v>12</v>
-      </c>
-      <c r="F60" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>16</v>
+      </c>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G60" s="13" t="inlineStr">
@@ -3221,23 +3221,23 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Designing with AI for Design Leaders</t>
+          <t>Ethics of AI in Design, Explained for B2B Teams</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>designing with ai</t>
+          <t>ethics of ai in design</t>
         </is>
       </c>
       <c r="D61" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E61" t="n">
-        <v>18</v>
-      </c>
-      <c r="F61" s="5" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>10</v>
+      </c>
+      <c r="F61" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G61" s="13" t="inlineStr">
@@ -3265,23 +3265,23 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>AI Design Process: What It Means for Your Brand</t>
+          <t>AI Web Design vs a Human Team: The Honest Trade-offs</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>ai design process</t>
+          <t>ai web design vs human</t>
         </is>
       </c>
       <c r="D62" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E62" t="n">
-        <v>16</v>
-      </c>
-      <c r="F62" s="5" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>12</v>
+      </c>
+      <c r="F62" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G62" s="13" t="inlineStr">
@@ -3300,94 +3300,6 @@
         </is>
       </c>
       <c r="J62" s="2" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Ethics of AI in Design, Explained for B2B Teams</t>
-        </is>
-      </c>
-      <c r="C63" s="3" t="inlineStr">
-        <is>
-          <t>ethics of ai in design</t>
-        </is>
-      </c>
-      <c r="D63" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E63" t="n">
-        <v>10</v>
-      </c>
-      <c r="F63" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
-        </is>
-      </c>
-      <c r="G63" s="13" t="inlineStr">
-        <is>
-          <t>AI + Human Thought Leadership</t>
-        </is>
-      </c>
-      <c r="H63" s="7" t="inlineStr">
-        <is>
-          <t>Early-mover bet</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>Top of funnel</t>
-        </is>
-      </c>
-      <c r="J63" s="2" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>AI Web Design vs a Human Team: The Honest Trade-offs</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="inlineStr">
-        <is>
-          <t>ai web design vs human</t>
-        </is>
-      </c>
-      <c r="D64" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E64" t="n">
-        <v>12</v>
-      </c>
-      <c r="F64" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
-        </is>
-      </c>
-      <c r="G64" s="13" t="inlineStr">
-        <is>
-          <t>AI + Human Thought Leadership</t>
-        </is>
-      </c>
-      <c r="H64" s="7" t="inlineStr">
-        <is>
-          <t>Early-mover bet</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>Top of funnel</t>
-        </is>
-      </c>
-      <c r="J64" s="2" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3874,9 +3786,9 @@
           <t>Demand now</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G14" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -4006,9 +3918,9 @@
           <t>Demand now</t>
         </is>
       </c>
-      <c r="G18" s="14" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G18" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -7910,7 +7822,7 @@
       <c r="A11" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  A · AI-Forward Positioning   (15 articles) — 'AI branding agency', 'AI web design agency', 'AI design subscription'. Mostly ~0 volume TODAY = early-mover bets to own the cluster when demand arrives in 1-2 months.
-  B · Fast &amp; Affordable Design (29 articles) — 'unlimited graphic design', 'web design subscription', 'low cost website design'. REAL demand now, and it maps exactly to your new faster / cost-efficient packages (SuperDesign). This is where traffic and leads come from in months 1-3.
+  B · Fast &amp; Affordable Design (27 articles) — 'unlimited graphic design', 'web design subscription', 'low cost website design'. REAL demand now, and it maps exactly to your new faster / cost-efficient packages (SuperDesign). This is where traffic and leads come from in months 1-3.
   C · AI + Human Thought Leadership (19 articles) — 'AI vs human designers', 'will AI replace web designers', 'AI in branding'. Evergreen positioning content that earns AI citations (AEO) and reassures buyers. Low volume, high authority value.</t>
         </is>
       </c>
@@ -7925,7 +7837,7 @@
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>Every article is tagged. 'Demand now' (31) = people search this today, expect ramp in months 2-4. 'Early-mover bet' (32) = ~0 volume today, published to own the term before competitors and before the demand curve. Average difficulty across the plan is just 20.0 — almost all easy wins.</t>
+          <t>Every article is tagged. 'Demand now' (29) = people search this today, expect ramp in months 2-4. 'Early-mover bet' (32) = ~0 volume today, published to own the term before competitors and before the demand curve. Average difficulty across the plan is just 20.0 — almost all easy wins.</t>
         </is>
       </c>
     </row>

</xml_diff>